<commit_message>
Relabel Pipeline sheet: recorded PRISMA counts, not estimates
</commit_message>
<xml_diff>
--- a/data/Taxonomy_Coding_Sheet_FINAL.xlsx
+++ b/data/Taxonomy_Coding_Sheet_FINAL.xlsx
@@ -5,18 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bastientogno/Desktop/Master Thesis/taxonomy/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bastientogno/Desktop/Master Thesis/open-sustainable-finance-data/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D2B159-BC0D-B140-A1ED-BB0310CC529F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAEFCA24-4AFD-AE49-B142-F1AB67A7DD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full Coding" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="7" r:id="rId2"/>
-    <sheet name="Codebook" sheetId="3" r:id="rId3"/>
-    <sheet name="Pipeline Estimate" sheetId="6" r:id="rId4"/>
+    <sheet name="Codebook" sheetId="3" r:id="rId2"/>
+    <sheet name="PRISMA Pipeline" sheetId="6" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Full Coding'!$A$2:$AG$111</definedName>
@@ -3456,9 +3455,6 @@
     <t>https://data.mendeley.com/datasets/b5f9rp823c/2</t>
   </si>
   <si>
-    <t>PIPELINE ESTIMATE  —  Rough count of papers in scope per journal</t>
-  </si>
-  <si>
     <t>ISSN</t>
   </si>
   <si>
@@ -3478,12 +3474,6 @@
     <t>1572-3097</t>
   </si>
   <si>
-    <t>ESTIMATED TOTAL</t>
-  </si>
-  <si>
-    <t>HOW TO VERIFY THESE ESTIMATES  —  Run the following Scopus search for each journal and replace estimates above</t>
-  </si>
-  <si>
     <t>Step 1 — Scopus search string (adapt per journal):</t>
   </si>
   <si>
@@ -3667,6 +3657,15 @@
   </si>
   <si>
     <t>Florida only</t>
+  </si>
+  <si>
+    <t>PIPELINE count of papers in scope per journal</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TOTAL</t>
+  </si>
+  <si>
+    <t>Search protocol</t>
   </si>
 </sst>
 </file>
@@ -4049,6 +4048,27 @@
     <xf numFmtId="0" fontId="12" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4079,8 +4099,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4097,25 +4115,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4474,52 +4473,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:33" ht="26" x14ac:dyDescent="0.2">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="42" t="s">
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="51" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="46" t="s">
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
+      <c r="J1" s="39"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="40"/>
+      <c r="Q1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="R1" s="47"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="36" t="s">
+      <c r="R1" s="54"/>
+      <c r="S1" s="40"/>
+      <c r="T1" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="U1" s="37"/>
-      <c r="V1" s="38"/>
-      <c r="W1" s="45" t="s">
+      <c r="U1" s="46"/>
+      <c r="V1" s="47"/>
+      <c r="W1" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="X1" s="43"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="48" t="s">
+      <c r="X1" s="39"/>
+      <c r="Y1" s="40"/>
+      <c r="Z1" s="55" t="s">
         <v>28</v>
       </c>
-      <c r="AA1" s="49"/>
-      <c r="AB1" s="39" t="s">
+      <c r="AA1" s="56"/>
+      <c r="AB1" s="48" t="s">
         <v>4</v>
       </c>
-      <c r="AC1" s="40"/>
-      <c r="AD1" s="40"/>
-      <c r="AE1" s="40"/>
-      <c r="AF1" s="41"/>
+      <c r="AC1" s="49"/>
+      <c r="AD1" s="49"/>
+      <c r="AE1" s="49"/>
+      <c r="AF1" s="50"/>
       <c r="AG1" s="7" t="s">
         <v>29</v>
       </c>
@@ -4553,7 +4552,7 @@
         <v>32</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>1041</v>
+        <v>1038</v>
       </c>
       <c r="K2" s="8" t="s">
         <v>33</v>
@@ -4580,16 +4579,16 @@
         <v>40</v>
       </c>
       <c r="S2" s="23" t="s">
-        <v>1050</v>
+        <v>1047</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>1042</v>
+        <v>1039</v>
       </c>
       <c r="U2" s="22" t="s">
         <v>151</v>
       </c>
       <c r="V2" s="24" t="s">
-        <v>1051</v>
+        <v>1048</v>
       </c>
       <c r="W2" s="4" t="s">
         <v>6</v>
@@ -4610,13 +4609,13 @@
         <v>43</v>
       </c>
       <c r="AC2" s="6" t="s">
-        <v>1052</v>
+        <v>1049</v>
       </c>
       <c r="AD2" s="6" t="s">
         <v>12</v>
       </c>
       <c r="AE2" s="6" t="s">
-        <v>1053</v>
+        <v>1050</v>
       </c>
       <c r="AF2" s="6" t="s">
         <v>254</v>
@@ -5019,7 +5018,7 @@
         <v>134</v>
       </c>
       <c r="AE7" s="10" t="s">
-        <v>1027</v>
+        <v>1024</v>
       </c>
       <c r="AF7" s="10"/>
       <c r="AG7" s="10" t="s">
@@ -5100,7 +5099,7 @@
         <v>134</v>
       </c>
       <c r="AE8" s="12" t="s">
-        <v>1028</v>
+        <v>1025</v>
       </c>
       <c r="AF8" s="12" t="s">
         <v>142</v>
@@ -5179,7 +5178,7 @@
         <v>134</v>
       </c>
       <c r="AE9" s="10" t="s">
-        <v>1029</v>
+        <v>1026</v>
       </c>
       <c r="AF9" s="10" t="s">
         <v>142</v>
@@ -5260,7 +5259,7 @@
         <v>134</v>
       </c>
       <c r="AE10" s="12" t="s">
-        <v>1030</v>
+        <v>1027</v>
       </c>
       <c r="AF10" s="12" t="s">
         <v>142</v>
@@ -5338,7 +5337,7 @@
         <v>381</v>
       </c>
       <c r="AB11" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC11" s="10" t="s">
         <v>382</v>
@@ -5347,7 +5346,7 @@
         <v>134</v>
       </c>
       <c r="AE11" s="10" t="s">
-        <v>1031</v>
+        <v>1028</v>
       </c>
       <c r="AF11" s="10" t="s">
         <v>142</v>
@@ -5428,7 +5427,7 @@
         <v>134</v>
       </c>
       <c r="AE12" s="12" t="s">
-        <v>1032</v>
+        <v>1029</v>
       </c>
       <c r="AF12" s="12" t="s">
         <v>150</v>
@@ -5507,7 +5506,7 @@
         <v>134</v>
       </c>
       <c r="AE13" s="10" t="s">
-        <v>1033</v>
+        <v>1030</v>
       </c>
       <c r="AF13" s="10" t="s">
         <v>150</v>
@@ -5524,7 +5523,7 @@
         <v>255</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>1048</v>
+        <v>1045</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>393</v>
@@ -5586,7 +5585,7 @@
         <v>134</v>
       </c>
       <c r="AE14" s="12" t="s">
-        <v>1034</v>
+        <v>1031</v>
       </c>
       <c r="AF14" s="12" t="s">
         <v>150</v>
@@ -5661,13 +5660,13 @@
         <v>142</v>
       </c>
       <c r="AC15" s="10" t="s">
-        <v>1026</v>
+        <v>1023</v>
       </c>
       <c r="AD15" s="10" t="s">
         <v>142</v>
       </c>
       <c r="AE15" s="10" t="s">
-        <v>1026</v>
+        <v>1023</v>
       </c>
       <c r="AF15" s="10" t="s">
         <v>142</v>
@@ -5752,7 +5751,7 @@
         <v>134</v>
       </c>
       <c r="AE16" s="12" t="s">
-        <v>1035</v>
+        <v>1032</v>
       </c>
       <c r="AF16" s="12" t="s">
         <v>142</v>
@@ -5901,7 +5900,7 @@
         <v>805</v>
       </c>
       <c r="AB18" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC18" s="12" t="s">
         <v>806</v>
@@ -5982,7 +5981,7 @@
         <v>810</v>
       </c>
       <c r="AB19" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC19" s="10" t="s">
         <v>811</v>
@@ -6064,13 +6063,13 @@
         <v>150</v>
       </c>
       <c r="AC20" s="12" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="AD20" s="12" t="s">
         <v>415</v>
       </c>
       <c r="AE20" s="12" t="s">
-        <v>1036</v>
+        <v>1033</v>
       </c>
       <c r="AF20" s="12" t="s">
         <v>150</v>
@@ -6142,7 +6141,7 @@
         <v>819</v>
       </c>
       <c r="AB21" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC21" s="10" t="s">
         <v>811</v>
@@ -6371,7 +6370,7 @@
         <v>830</v>
       </c>
       <c r="AB24" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC24" s="12" t="s">
         <v>831</v>
@@ -6606,7 +6605,7 @@
         <v>699</v>
       </c>
       <c r="AB27" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC27" s="10" t="s">
         <v>842</v>
@@ -6766,7 +6765,7 @@
         <v>850</v>
       </c>
       <c r="AB29" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC29" s="10" t="s">
         <v>851</v>
@@ -6888,7 +6887,7 @@
       <c r="N31" s="21"/>
       <c r="O31" s="21"/>
       <c r="P31" s="21" t="s">
-        <v>1040</v>
+        <v>1037</v>
       </c>
       <c r="Q31" s="10" t="s">
         <v>296</v>
@@ -6922,7 +6921,7 @@
         <v>859</v>
       </c>
       <c r="AB31" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC31" s="10" t="s">
         <v>860</v>
@@ -7467,7 +7466,7 @@
         <v>928</v>
       </c>
       <c r="AB38" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC38" s="12" t="s">
         <v>969</v>
@@ -7548,7 +7547,7 @@
         <v>930</v>
       </c>
       <c r="AB39" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC39" s="10" t="s">
         <v>971</v>
@@ -7789,7 +7788,7 @@
         <v>935</v>
       </c>
       <c r="AB42" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC42" s="12" t="s">
         <v>970</v>
@@ -7870,7 +7869,7 @@
         <v>693</v>
       </c>
       <c r="AB43" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC43" s="10" t="s">
         <v>973</v>
@@ -8869,7 +8868,7 @@
       <c r="N56" s="21"/>
       <c r="O56" s="21"/>
       <c r="P56" s="21" t="s">
-        <v>1023</v>
+        <v>1020</v>
       </c>
       <c r="Q56" s="12" t="s">
         <v>296</v>
@@ -9055,7 +9054,7 @@
         <v>967</v>
       </c>
       <c r="AB58" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC58" s="12" t="s">
         <v>968</v>
@@ -9298,7 +9297,7 @@
         <v>420</v>
       </c>
       <c r="AB61" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC61" s="10" t="s">
         <v>421</v>
@@ -9379,7 +9378,7 @@
         <v>425</v>
       </c>
       <c r="AB62" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC62" s="12" t="s">
         <v>426</v>
@@ -9568,7 +9567,7 @@
         <v>439</v>
       </c>
       <c r="F65" s="10" t="s">
-        <v>1037</v>
+        <v>1034</v>
       </c>
       <c r="G65" s="21"/>
       <c r="H65" s="21"/>
@@ -9620,7 +9619,7 @@
         <v>441</v>
       </c>
       <c r="AB65" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC65" s="10" t="s">
         <v>442</v>
@@ -9854,7 +9853,7 @@
         <v>140</v>
       </c>
       <c r="AA68" s="12" t="s">
-        <v>1054</v>
+        <v>1051</v>
       </c>
       <c r="AB68" s="12" t="s">
         <v>150</v>
@@ -10092,7 +10091,7 @@
         <v>596</v>
       </c>
       <c r="AB71" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC71" s="10" t="s">
         <v>597</v>
@@ -10175,7 +10174,7 @@
         <v>601</v>
       </c>
       <c r="AB72" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC72" s="12" t="s">
         <v>602</v>
@@ -10254,7 +10253,7 @@
         <v>606</v>
       </c>
       <c r="AB73" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC73" s="10" t="s">
         <v>607</v>
@@ -10651,7 +10650,7 @@
         <v>633</v>
       </c>
       <c r="AB78" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC78" s="12" t="s">
         <v>634</v>
@@ -10734,7 +10733,7 @@
         <v>638</v>
       </c>
       <c r="AB79" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC79" s="10" t="s">
         <v>639</v>
@@ -10890,7 +10889,7 @@
         <v>648</v>
       </c>
       <c r="AB81" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC81" s="10" t="s">
         <v>649</v>
@@ -11052,7 +11051,7 @@
       <c r="AB83" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="AC83" s="56" t="s">
+      <c r="AC83" s="33" t="s">
         <v>148</v>
       </c>
       <c r="AD83" s="10" t="s">
@@ -11082,7 +11081,7 @@
       <c r="E84" s="12" t="s">
         <v>660</v>
       </c>
-      <c r="F84" s="57" t="s">
+      <c r="F84" s="34" t="s">
         <v>144</v>
       </c>
       <c r="G84" s="21"/>
@@ -11113,7 +11112,7 @@
         <v>297</v>
       </c>
       <c r="V84" s="12" t="s">
-        <v>1056</v>
+        <v>1053</v>
       </c>
       <c r="W84" s="12">
         <v>2026</v>
@@ -11128,7 +11127,7 @@
         <v>143</v>
       </c>
       <c r="AA84" s="12" t="s">
-        <v>1057</v>
+        <v>1054</v>
       </c>
       <c r="AB84" s="12" t="s">
         <v>134</v>
@@ -11453,7 +11452,7 @@
         <v>678</v>
       </c>
       <c r="AB88" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC88" s="12" t="s">
         <v>679</v>
@@ -11531,10 +11530,10 @@
         <v>143</v>
       </c>
       <c r="AA89" s="10" t="s">
-        <v>1021</v>
+        <v>1018</v>
       </c>
       <c r="AB89" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC89" s="10" t="s">
         <v>683</v>
@@ -11615,7 +11614,7 @@
         <v>687</v>
       </c>
       <c r="AB90" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC90" s="12" t="s">
         <v>688</v>
@@ -11696,7 +11695,7 @@
         <v>693</v>
       </c>
       <c r="AB91" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC91" s="10" t="s">
         <v>694</v>
@@ -11773,7 +11772,7 @@
         <v>699</v>
       </c>
       <c r="AB92" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC92" s="12" t="s">
         <v>700</v>
@@ -11856,7 +11855,7 @@
       <c r="AB93" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="AC93" s="56" t="s">
+      <c r="AC93" s="33" t="s">
         <v>705</v>
       </c>
       <c r="AD93" s="10" t="s">
@@ -11933,7 +11932,7 @@
         <v>709</v>
       </c>
       <c r="AB94" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC94" s="12" t="s">
         <v>710</v>
@@ -12089,7 +12088,7 @@
         <v>719</v>
       </c>
       <c r="AB96" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC96" s="12" t="s">
         <v>720</v>
@@ -12403,7 +12402,7 @@
         <v>736</v>
       </c>
       <c r="AB100" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC100" s="12" t="s">
         <v>737</v>
@@ -12484,7 +12483,7 @@
         <v>740</v>
       </c>
       <c r="AB101" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC101" s="10" t="s">
         <v>742</v>
@@ -12567,7 +12566,7 @@
         <v>747</v>
       </c>
       <c r="AB102" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC102" s="12" t="s">
         <v>748</v>
@@ -12614,7 +12613,7 @@
         <v>134</v>
       </c>
       <c r="P103" s="21" t="s">
-        <v>1024</v>
+        <v>1021</v>
       </c>
       <c r="Q103" s="10" t="s">
         <v>66</v>
@@ -12727,7 +12726,7 @@
         <v>758</v>
       </c>
       <c r="AB104" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC104" s="12" t="s">
         <v>759</v>
@@ -12810,7 +12809,7 @@
         <v>764</v>
       </c>
       <c r="AB105" s="10" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC105" s="10" t="s">
         <v>766</v>
@@ -12859,7 +12858,7 @@
       <c r="N106" s="21"/>
       <c r="O106" s="21"/>
       <c r="P106" s="21" t="s">
-        <v>1025</v>
+        <v>1022</v>
       </c>
       <c r="Q106" s="12" t="s">
         <v>296</v>
@@ -12893,7 +12892,7 @@
         <v>770</v>
       </c>
       <c r="AB106" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC106" s="12" t="s">
         <v>771</v>
@@ -12973,7 +12972,7 @@
         <v>139</v>
       </c>
       <c r="AA107" s="10" t="s">
-        <v>1055</v>
+        <v>1052</v>
       </c>
       <c r="AB107" s="10" t="s">
         <v>142</v>
@@ -13057,7 +13056,7 @@
         <v>780</v>
       </c>
       <c r="AB108" s="12" t="s">
-        <v>1022</v>
+        <v>1019</v>
       </c>
       <c r="AC108" s="12" t="s">
         <v>781</v>
@@ -13400,15 +13399,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2AE3150F-1356-2444-B1FC-75F36F3DC5BB}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -13419,11 +13409,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="57" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
@@ -13438,13 +13428,13 @@
     </row>
     <row r="3" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="15" t="s">
-        <v>1038</v>
+        <v>1035</v>
       </c>
       <c r="B3" s="16" t="s">
         <v>116</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>1039</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="32" customHeight="1" x14ac:dyDescent="0.2">
@@ -13804,7 +13794,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2270F5D0-6006-FF49-B46C-78789857AC63}">
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -13818,33 +13808,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="52" t="s">
-        <v>988</v>
-      </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
+      <c r="A1" s="35" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
     </row>
     <row r="2" spans="1:6" ht="49" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>118</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="C2" s="14" t="s">
         <v>119</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>120</v>
       </c>
       <c r="F2" s="14" t="s">
-        <v>1043</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -13852,7 +13842,7 @@
         <v>122</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="C3" s="10">
         <v>18</v>
@@ -13864,7 +13854,7 @@
         <v>14</v>
       </c>
       <c r="F3" s="31" t="s">
-        <v>1046</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -13872,7 +13862,7 @@
         <v>123</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="C4" s="12">
         <v>57</v>
@@ -13884,7 +13874,7 @@
         <v>42</v>
       </c>
       <c r="F4" s="32" t="s">
-        <v>1044</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -13892,7 +13882,7 @@
         <v>124</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="C5" s="10">
         <v>30</v>
@@ -13904,7 +13894,7 @@
         <v>22</v>
       </c>
       <c r="F5" s="31" t="s">
-        <v>1045</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -13912,7 +13902,7 @@
         <v>125</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C6" s="12">
         <v>42</v>
@@ -13924,12 +13914,12 @@
         <v>31</v>
       </c>
       <c r="F6" s="32" t="s">
-        <v>1047</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="25" t="s">
-        <v>995</v>
+        <v>1056</v>
       </c>
       <c r="B7" s="26"/>
       <c r="C7" s="26">
@@ -13945,7 +13935,7 @@
         <v>109</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>1049</v>
+        <v>1046</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -13956,45 +13946,45 @@
       <c r="E8" s="27"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" s="53" t="s">
-        <v>996</v>
-      </c>
-      <c r="B9" s="51"/>
-      <c r="C9" s="51"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
+      <c r="A9" s="36" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B9" s="37"/>
+      <c r="C9" s="37"/>
+      <c r="D9" s="37"/>
+      <c r="E9" s="37"/>
     </row>
     <row r="10" spans="1:6" ht="219" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="28" t="s">
-        <v>997</v>
-      </c>
-      <c r="B10" s="54" t="s">
-        <v>1020</v>
-      </c>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="44"/>
+        <v>994</v>
+      </c>
+      <c r="B10" s="38" t="s">
+        <v>1017</v>
+      </c>
+      <c r="C10" s="39"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="40"/>
     </row>
     <row r="11" spans="1:6" ht="79" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="29" t="s">
-        <v>998</v>
-      </c>
-      <c r="B11" s="55" t="s">
-        <v>999</v>
-      </c>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="44"/>
+        <v>995</v>
+      </c>
+      <c r="B11" s="41" t="s">
+        <v>996</v>
+      </c>
+      <c r="C11" s="39"/>
+      <c r="D11" s="39"/>
+      <c r="E11" s="40"/>
     </row>
     <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="53" t="s">
-        <v>1000</v>
-      </c>
-      <c r="B13" s="51"/>
-      <c r="C13" s="51"/>
-      <c r="D13" s="51"/>
-      <c r="E13" s="51"/>
+      <c r="A13" s="36" t="s">
+        <v>997</v>
+      </c>
+      <c r="B13" s="37"/>
+      <c r="C13" s="37"/>
+      <c r="D13" s="37"/>
+      <c r="E13" s="37"/>
     </row>
     <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="17" t="s">
@@ -14004,7 +13994,7 @@
         <v>127</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>1001</v>
+        <v>998</v>
       </c>
       <c r="D14" s="18" t="s">
         <v>128</v>
@@ -14018,16 +14008,16 @@
         <v>129</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>999</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>1001</v>
+      </c>
+      <c r="E15" s="11" t="s">
         <v>1002</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>1003</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>1004</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>1005</v>
       </c>
     </row>
     <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
@@ -14035,30 +14025,30 @@
         <v>130</v>
       </c>
       <c r="B16" s="12" t="s">
+        <v>1003</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>1004</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E16" s="13" t="s">
         <v>1006</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>1007</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>1008</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>1009</v>
       </c>
     </row>
     <row r="17" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="11" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>1008</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>1009</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>1010</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>1011</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>1012</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>1013</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>131</v>
@@ -14069,16 +14059,16 @@
         <v>132</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>1015</v>
+        <v>1012</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>1016</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="19" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
@@ -14086,30 +14076,30 @@
         <v>133</v>
       </c>
       <c r="B19" s="10" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>1011</v>
+      </c>
+      <c r="D19" s="10" t="s">
         <v>1014</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>1014</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>1017</v>
-      </c>
       <c r="E19" s="11" t="s">
-        <v>1016</v>
+        <v>1013</v>
       </c>
     </row>
     <row r="20" spans="1:5" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="25" t="s">
-        <v>1018</v>
+        <v>1015</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>1014</v>
+        <v>1011</v>
       </c>
       <c r="D20" s="26" t="s">
-        <v>1019</v>
+        <v>1016</v>
       </c>
       <c r="E20" s="25"/>
     </row>

</xml_diff>